<commit_message>
Updates for Bolivian run
Minor updates and changes were made to scripts and control files to re-run the Bolivian case
</commit_message>
<xml_diff>
--- a/1. MSR Creator/ControlFile_MSRCreator.xlsx
+++ b/1. MSR Creator/ControlFile_MSRCreator.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Carlos\Desktop\MSR\Model-Supply-Regions-MSR-Toolset\1. MSR Creator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7F023BA0-03A8-4520-93A5-BA2B32C98289}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFEDC9F6-26D1-48C5-AF8A-1DF9660EAA2D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="23880" yWindow="-6870" windowWidth="29040" windowHeight="15720" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Paths" sheetId="9" r:id="rId1"/>
@@ -71,7 +71,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="181">
   <si>
     <t>Parameter</t>
   </si>
@@ -610,7 +610,10 @@
     <t>C:\Users\Carlos\Desktop\MSR\Model-Supply-Regions-MSR-Toolset\countrynames.csv</t>
   </si>
   <si>
-    <t>wind</t>
+    <t>Pixels below this value will be disregarded. Value can be changed by code if iterative relaxer mode is on. Units: kWh/m2-day (****initially 4, but changed to include more surface)</t>
+  </si>
+  <si>
+    <t>solarpv</t>
   </si>
 </sst>
 </file>
@@ -1178,7 +1181,7 @@
         <v>23</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>24</v>
@@ -2308,10 +2311,10 @@
         <v>116</v>
       </c>
       <c r="B2" s="6">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>117</v>
+        <v>179</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -2385,10 +2388,10 @@
         <v>127</v>
       </c>
       <c r="B9" s="6">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>128</v>
+        <v>174</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">

</xml_diff>